<commit_message>
fix(data): correct HENU-ACMERDB source data by @Envystar
</commit_message>
<xml_diff>
--- a/HENU-ACMERDB.xlsx
+++ b/HENU-ACMERDB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Enar\VSCode\project\HENU-ACMERDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB50989A-9F3A-48E8-831C-F3078FC62AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83C7C2DF-A818-431A-971A-594B2B5A268C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="4" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="546">
   <si>
     <t>比赛类型</t>
   </si>
@@ -1670,6 +1670,9 @@
   </si>
   <si>
     <t>李硕,赵紫林,韩中贤</t>
+  </si>
+  <si>
+    <t>李想, 吴逸轩, 献超前</t>
   </si>
 </sst>
 </file>
@@ -4468,25 +4471,25 @@
         <v>196</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>139</v>
+        <v>31</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>197</v>
+        <v>32</v>
       </c>
       <c r="E46" s="16" t="s">
         <v>33</v>
       </c>
       <c r="F46" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G46" s="4">
-        <v>125</v>
+        <v>311</v>
       </c>
       <c r="H46" s="16">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="I46" s="16">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="J46" s="16" t="s">
         <v>6</v>
@@ -4495,7 +4498,7 @@
         <v>7</v>
       </c>
       <c r="L46" s="16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M46" s="17"/>
       <c r="N46" s="1"/>
@@ -4524,22 +4527,22 @@
         <v>196</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>31</v>
+        <v>139</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>32</v>
+        <v>197</v>
       </c>
       <c r="E47" s="16" t="s">
         <v>33</v>
       </c>
       <c r="F47" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G47" s="4">
-        <v>158</v>
+        <v>625</v>
       </c>
       <c r="H47" s="16">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="I47" s="16" t="s">
         <v>34</v>
@@ -4583,19 +4586,19 @@
         <v>152</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>32</v>
+        <v>545</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F48" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G48" s="4">
-        <v>137</v>
+        <v>485</v>
       </c>
       <c r="H48" s="16">
-        <v>363</v>
+        <v>327</v>
       </c>
       <c r="I48" s="16" t="s">
         <v>34</v>

</xml_diff>